<commit_message>
feat(abc): lock cells with sheet password (only Qtd./Custo/limites editaveis)
Each ABC tab and the Dashboard ship protected so the formulas stay
intact. Only the editable cells stay unlocked:

  - E and F (Qtd. and Custo Unit.) across the whole data range
  - B9 and B10 (ABC limits)

Password: "reggae" - editable at the top of build_abc.py
(PROTECTION_PASSWORD constant) for users who want a different one.

The comment on E12/F12 now tells the user how to unprotect the sheet
and what the password is.
</commit_message>
<xml_diff>
--- a/output/curva_abc_reggae_6.xlsx
+++ b/output/curva_abc_reggae_6.xlsx
@@ -2111,14 +2111,18 @@
     </comment>
     <comment ref="E12" authorId="1" shapeId="0">
       <text>
-        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.).
-V.T., % e Classe ABC sao recalculados automaticamente.</t>
+        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.) - elas estao
+desbloqueadas. V.T., % e Classe ABC recalculam automaticamente.
+Para desproteger a aba: Revisao -&gt; Desproteger Planilha
+Senha: reggae</t>
       </text>
     </comment>
     <comment ref="F12" authorId="1" shapeId="0">
       <text>
-        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.).
-V.T., % e Classe ABC sao recalculados automaticamente.</t>
+        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.) - elas estao
+desbloqueadas. V.T., % e Classe ABC recalculam automaticamente.
+Para desproteger a aba: Revisao -&gt; Desproteger Planilha
+Senha: reggae</t>
       </text>
     </comment>
   </commentList>
@@ -2148,14 +2152,18 @@
     </comment>
     <comment ref="E12" authorId="1" shapeId="0">
       <text>
-        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.).
-V.T., % e Classe ABC sao recalculados automaticamente.</t>
+        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.) - elas estao
+desbloqueadas. V.T., % e Classe ABC recalculam automaticamente.
+Para desproteger a aba: Revisao -&gt; Desproteger Planilha
+Senha: reggae</t>
       </text>
     </comment>
     <comment ref="F12" authorId="1" shapeId="0">
       <text>
-        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.).
-V.T., % e Classe ABC sao recalculados automaticamente.</t>
+        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.) - elas estao
+desbloqueadas. V.T., % e Classe ABC recalculam automaticamente.
+Para desproteger a aba: Revisao -&gt; Desproteger Planilha
+Senha: reggae</t>
       </text>
     </comment>
   </commentList>
@@ -2185,14 +2193,18 @@
     </comment>
     <comment ref="E12" authorId="1" shapeId="0">
       <text>
-        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.).
-V.T., % e Classe ABC sao recalculados automaticamente.</t>
+        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.) - elas estao
+desbloqueadas. V.T., % e Classe ABC recalculam automaticamente.
+Para desproteger a aba: Revisao -&gt; Desproteger Planilha
+Senha: reggae</t>
       </text>
     </comment>
     <comment ref="F12" authorId="1" shapeId="0">
       <text>
-        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.).
-V.T., % e Classe ABC sao recalculados automaticamente.</t>
+        <t>Edite apenas as colunas E (Qtd.) e F (Custo Unit.) - elas estao
+desbloqueadas. V.T., % e Classe ABC recalculam automaticamente.
+Para desproteger a aba: Revisao -&gt; Desproteger Planilha
+Senha: reggae</t>
       </text>
     </comment>
   </commentList>
@@ -3086,6 +3098,7 @@
       <c r="K43" s="75" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF15"/>
   <mergeCells count="7">
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="B9:K9"/>
@@ -4386,7 +4399,7 @@
     </row>
     <row r="23" ht="18" customHeight="1"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="F0B1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF15"/>
   <mergeCells count="21">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A22:D22"/>
@@ -6627,7 +6640,7 @@
     </row>
     <row r="33" ht="18" customHeight="1"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="F0B1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF15"/>
   <mergeCells count="21">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C5:D5"/>
@@ -9748,7 +9761,7 @@
     </row>
     <row r="43" ht="18" customHeight="1"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="F0B1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF15"/>
   <mergeCells count="21">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C5:D5"/>

</xml_diff>